<commit_message>
fix(kashmir): realistic per-route population on the map + table
The network-map popup showed the apportioned corridor share (~262 people),
which looked unrealistically small. It now shows Population_Served_Raw — the
400m walkshed population (~70k), the intuitive "people along this route" figure
— and the real Route_Code (the geojson now carries both). The route table's
"Population served" sort uses the same walkshed figure.

- lib: added populationServedRaw to the route type + normalizer.
- Refreshed geojson + pretty/RTO workbooks from the v3.3.7 re-run.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.3.7_RTO.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.3.7_RTO.xlsx
@@ -883,7 +883,7 @@
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Version: v3.3.7  |  Generated: 29 May 2026</t>
+          <t>Version: v3.3.7  |  Generated: 30 May 2026</t>
         </is>
       </c>
     </row>
@@ -45437,7 +45437,7 @@
       </c>
       <c r="C5" s="75" t="inlineStr">
         <is>
-          <t>29 May 2026</t>
+          <t>30 May 2026</t>
         </is>
       </c>
     </row>

</xml_diff>